<commit_message>
Update Confronto Metriche - 18Mag26.xlsx
</commit_message>
<xml_diff>
--- a/PythonProject/results/Confronto Metriche - 18Mag26.xlsx
+++ b/PythonProject/results/Confronto Metriche - 18Mag26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t_789\Desktop\Sviluppo\ML_4_VIsion_-_Multimedia\PythonProject\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7850EC19-B7DF-43E4-8812-45BB67E58F5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB6C3771-1C95-4B60-AA46-3CF449A11AFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="279">
   <si>
     <t>Loss</t>
   </si>
@@ -76,9 +76,6 @@
     <t>Recall@100</t>
   </si>
   <si>
-    <t>0.11745113614033731</t>
-  </si>
-  <si>
     <t>0.5705702734272173</t>
   </si>
   <si>
@@ -121,9 +118,6 @@
     <t>0.8559582800511513</t>
   </si>
   <si>
-    <t>0.13738856774401817</t>
-  </si>
-  <si>
     <t>0.5221875954191004</t>
   </si>
   <si>
@@ -136,9 +130,6 @@
     <t>0.7496666666666667</t>
   </si>
   <si>
-    <t>0.49228576865147117</t>
-  </si>
-  <si>
     <t>0.5810461619313849</t>
   </si>
   <si>
@@ -163,36 +154,18 @@
     <t>Recall@200</t>
   </si>
   <si>
-    <t>0.08692697923138928</t>
-  </si>
-  <si>
     <t>0.6956154413079105</t>
   </si>
   <si>
-    <t>Dataset - E5 - M05 - LR000003</t>
-  </si>
-  <si>
-    <t>Dataset - E5 - M06 - LR2.5e-6</t>
-  </si>
-  <si>
     <t>0.6462941235068799</t>
   </si>
   <si>
-    <t>Dataset - E5 - M06 - LR</t>
-  </si>
-  <si>
-    <t>Dataset - E5 - M06 - LR000001</t>
-  </si>
-  <si>
     <t>0.2540397051932474</t>
   </si>
   <si>
     <t>0.3918033701054625</t>
   </si>
   <si>
-    <t>0.9139683123046961</t>
-  </si>
-  <si>
     <t>0.8966666666666666</t>
   </si>
   <si>
@@ -205,24 +178,15 @@
     <t>0.3857225044777708</t>
   </si>
   <si>
-    <t>0.45319766303592957</t>
-  </si>
-  <si>
     <t>0.509211822073637</t>
   </si>
   <si>
     <t>0.6281626334123572</t>
   </si>
   <si>
-    <t>0.9696428571428571</t>
-  </si>
-  <si>
     <t>0.96875</t>
   </si>
   <si>
-    <t>0.9187500000000001</t>
-  </si>
-  <si>
     <t>0.5003161144405848</t>
   </si>
   <si>
@@ -232,7 +196,676 @@
     <t>0.7564865092695094</t>
   </si>
   <si>
-    <t>Dataset - E5 - M06 - LR0000001</t>
+    <t>Dataset - E10 - M04 - LR000025. - 11_05_2026</t>
+  </si>
+  <si>
+    <t>0.0594315928896659</t>
+  </si>
+  <si>
+    <t>0.5905230985028451</t>
+  </si>
+  <si>
+    <t>0.9375880084934634</t>
+  </si>
+  <si>
+    <t>0.9233333333333332</t>
+  </si>
+  <si>
+    <t>0.8440000000000001</t>
+  </si>
+  <si>
+    <t>0.7750000000000004</t>
+  </si>
+  <si>
+    <t>0.5367515834409474</t>
+  </si>
+  <si>
+    <t>0.6328362184507096</t>
+  </si>
+  <si>
+    <t>0.6987054318122994</t>
+  </si>
+  <si>
+    <t>0.7030001876292077</t>
+  </si>
+  <si>
+    <t>0.9188022575250836</t>
+  </si>
+  <si>
+    <t>0.8625</t>
+  </si>
+  <si>
+    <t>0.84375</t>
+  </si>
+  <si>
+    <t>0.5397051666221323</t>
+  </si>
+  <si>
+    <t>0.733402600170503</t>
+  </si>
+  <si>
+    <t>0.847672900682012</t>
+  </si>
+  <si>
+    <t>Dataset - E10 - M04 - LR000025. - 13_05_2026</t>
+  </si>
+  <si>
+    <t>0.0828407202074759</t>
+  </si>
+  <si>
+    <t>0.491846485219114</t>
+  </si>
+  <si>
+    <t>0.9209890555255942</t>
+  </si>
+  <si>
+    <t>0.9033333333333332</t>
+  </si>
+  <si>
+    <t>0.7946666666666666</t>
+  </si>
+  <si>
+    <t>0.7126666666666669</t>
+  </si>
+  <si>
+    <t>0.4691549717033831</t>
+  </si>
+  <si>
+    <t>0.5587717162096626</t>
+  </si>
+  <si>
+    <t>0.6246931732591983</t>
+  </si>
+  <si>
+    <t>0.56585494407234</t>
+  </si>
+  <si>
+    <t>0.9291666666666666</t>
+  </si>
+  <si>
+    <t>0.8062500000000001</t>
+  </si>
+  <si>
+    <t>0.7531249999999998</t>
+  </si>
+  <si>
+    <t>0.435971417687776</t>
+  </si>
+  <si>
+    <t>0.6282298346820882</t>
+  </si>
+  <si>
+    <t>0.7750559462915603</t>
+  </si>
+  <si>
+    <t>Dataset - E10 - M04 - LR00005.</t>
+  </si>
+  <si>
+    <t>0.0872068546326854</t>
+  </si>
+  <si>
+    <t>0.4472390717800812</t>
+  </si>
+  <si>
+    <t>0.8925707233269001</t>
+  </si>
+  <si>
+    <t>0.8633333333333333</t>
+  </si>
+  <si>
+    <t>0.7286666666666662</t>
+  </si>
+  <si>
+    <t>0.6583333333333338</t>
+  </si>
+  <si>
+    <t>0.4421113826247222</t>
+  </si>
+  <si>
+    <t>0.5328103925514679</t>
+  </si>
+  <si>
+    <t>0.6081325295271285</t>
+  </si>
+  <si>
+    <t>0.5025801310809269</t>
+  </si>
+  <si>
+    <t>0.8358031988907669</t>
+  </si>
+  <si>
+    <t>0.8125</t>
+  </si>
+  <si>
+    <t>0.74375</t>
+  </si>
+  <si>
+    <t>0.6750000000000002</t>
+  </si>
+  <si>
+    <t>0.3906216201600692</t>
+  </si>
+  <si>
+    <t>0.55841705395656</t>
+  </si>
+  <si>
+    <t>0.6902307118499574</t>
+  </si>
+  <si>
+    <t>Dataset - E5 - M04 - LR00005.</t>
+  </si>
+  <si>
+    <t>0.0914351398791495</t>
+  </si>
+  <si>
+    <t>0.4408826875251142</t>
+  </si>
+  <si>
+    <t>0.9023559032496108</t>
+  </si>
+  <si>
+    <t>0.8866666666666667</t>
+  </si>
+  <si>
+    <t>0.7433333333333333</t>
+  </si>
+  <si>
+    <t>0.6593333333333335</t>
+  </si>
+  <si>
+    <t>0.4348022380819724</t>
+  </si>
+  <si>
+    <t>0.524835411198085</t>
+  </si>
+  <si>
+    <t>0.5948914522480889</t>
+  </si>
+  <si>
+    <t>0.4631288517713047</t>
+  </si>
+  <si>
+    <t>0.740185446946682</t>
+  </si>
+  <si>
+    <t>0.65625</t>
+  </si>
+  <si>
+    <t>0.6749999999999999</t>
+  </si>
+  <si>
+    <t>0.6375000000000001</t>
+  </si>
+  <si>
+    <t>0.3639006056673157</t>
+  </si>
+  <si>
+    <t>0.5063405797101449</t>
+  </si>
+  <si>
+    <t>0.6245471014492754</t>
+  </si>
+  <si>
+    <t>Dataset - E10 - M05 - LR000025. - 12_05_2026</t>
+  </si>
+  <si>
+    <t>0.0709138296330758</t>
+  </si>
+  <si>
+    <t>0.6079354018422084</t>
+  </si>
+  <si>
+    <t>0.9314370098871494</t>
+  </si>
+  <si>
+    <t>0.9133333333333332</t>
+  </si>
+  <si>
+    <t>0.8300000000000002</t>
+  </si>
+  <si>
+    <t>0.7660000000000003</t>
+  </si>
+  <si>
+    <t>0.5539225437617674</t>
+  </si>
+  <si>
+    <t>0.6568080597894279</t>
+  </si>
+  <si>
+    <t>0.726256729288847</t>
+  </si>
+  <si>
+    <t>0.6640369659648535</t>
+  </si>
+  <si>
+    <t>0.845807017107619</t>
+  </si>
+  <si>
+    <t>0.8250000000000001</t>
+  </si>
+  <si>
+    <t>0.5129308699469405</t>
+  </si>
+  <si>
+    <t>0.7029915957297912</t>
+  </si>
+  <si>
+    <t>0.7945705456095481</t>
+  </si>
+  <si>
+    <t>Dataset - E5 - M05 - LR000025.</t>
+  </si>
+  <si>
+    <t>0.0764052240601327</t>
+  </si>
+  <si>
+    <t>0.5824100348937288</t>
+  </si>
+  <si>
+    <t>0.9252278422558204</t>
+  </si>
+  <si>
+    <t>0.9066666666666666</t>
+  </si>
+  <si>
+    <t>0.811333333333333</t>
+  </si>
+  <si>
+    <t>0.7450000000000006</t>
+  </si>
+  <si>
+    <t>0.5364146365999661</t>
+  </si>
+  <si>
+    <t>0.6362746365566136</t>
+  </si>
+  <si>
+    <t>0.7118641191508265</t>
+  </si>
+  <si>
+    <t>0.6581412250315876</t>
+  </si>
+  <si>
+    <t>0.914906754032258</t>
+  </si>
+  <si>
+    <t>0.8531249999999999</t>
+  </si>
+  <si>
+    <t>0.4966331823936582</t>
+  </si>
+  <si>
+    <t>0.6839767156862745</t>
+  </si>
+  <si>
+    <t>0.8000186487638534</t>
+  </si>
+  <si>
+    <t>Dataset - E10 - M05 - LR000025. - 13_05_2026</t>
+  </si>
+  <si>
+    <t>0.1170190745204962</t>
+  </si>
+  <si>
+    <t>0.4587856302165331</t>
+  </si>
+  <si>
+    <t>0.8988880467988666</t>
+  </si>
+  <si>
+    <t>0.88</t>
+  </si>
+  <si>
+    <t>0.7566666666666668</t>
+  </si>
+  <si>
+    <t>0.6773333333333331</t>
+  </si>
+  <si>
+    <t>0.448220578354971</t>
+  </si>
+  <si>
+    <t>0.5392127798409377</t>
+  </si>
+  <si>
+    <t>0.6154774418482699</t>
+  </si>
+  <si>
+    <t>0.5756013733734875</t>
+  </si>
+  <si>
+    <t>0.8800223214285714</t>
+  </si>
+  <si>
+    <t>0.771875</t>
+  </si>
+  <si>
+    <t>0.4540673788983471</t>
+  </si>
+  <si>
+    <t>0.6182731244671782</t>
+  </si>
+  <si>
+    <t>0.7283807544757033</t>
+  </si>
+  <si>
+    <t>Dataset - E5 - M05 - LR0000001.</t>
+  </si>
+  <si>
+    <t>0.2158000818112128</t>
+  </si>
+  <si>
+    <t>0.3739158361736051</t>
+  </si>
+  <si>
+    <t>0.911269258972538</t>
+  </si>
+  <si>
+    <t>0.89</t>
+  </si>
+  <si>
+    <t>0.7319999999999999</t>
+  </si>
+  <si>
+    <t>0.6423333333333338</t>
+  </si>
+  <si>
+    <t>0.3763412258967861</t>
+  </si>
+  <si>
+    <t>0.4433451587917529</t>
+  </si>
+  <si>
+    <t>0.5005893967160635</t>
+  </si>
+  <si>
+    <t>0.6222531001974437</t>
+  </si>
+  <si>
+    <t>0.9696969696969696</t>
+  </si>
+  <si>
+    <t>0.9125</t>
+  </si>
+  <si>
+    <t>0.890625</t>
+  </si>
+  <si>
+    <t>0.498950758515606</t>
+  </si>
+  <si>
+    <t>0.6463387188100418</t>
+  </si>
+  <si>
+    <t>0.7623743892430432</t>
+  </si>
+  <si>
+    <t>Dataset - E5 - M05 - LR00000025.</t>
+  </si>
+  <si>
+    <t>0.1674994876697035</t>
+  </si>
+  <si>
+    <t>0.4332957508495203</t>
+  </si>
+  <si>
+    <t>0.9276166930616034</t>
+  </si>
+  <si>
+    <t>0.91</t>
+  </si>
+  <si>
+    <t>0.7786666666666668</t>
+  </si>
+  <si>
+    <t>0.6910000000000002</t>
+  </si>
+  <si>
+    <t>0.4228432556730581</t>
+  </si>
+  <si>
+    <t>0.4936394605972914</t>
+  </si>
+  <si>
+    <t>0.5525235941879927</t>
+  </si>
+  <si>
+    <t>0.6641580941246649</t>
+  </si>
+  <si>
+    <t>0.9534471649484536</t>
+  </si>
+  <si>
+    <t>0.94375</t>
+  </si>
+  <si>
+    <t>0.909375</t>
+  </si>
+  <si>
+    <t>0.5206967480373069</t>
+  </si>
+  <si>
+    <t>0.6812724461134226</t>
+  </si>
+  <si>
+    <t>0.7859521526001708</t>
+  </si>
+  <si>
+    <t>Dataset - E5 - M05 - LR000001.</t>
+  </si>
+  <si>
+    <t>0.1145220818421837</t>
+  </si>
+  <si>
+    <t>0.5061790567456045</t>
+  </si>
+  <si>
+    <t>0.9368281283658738</t>
+  </si>
+  <si>
+    <t>0.8166666666666665</t>
+  </si>
+  <si>
+    <t>0.7403333333333332</t>
+  </si>
+  <si>
+    <t>0.4801643544923956</t>
+  </si>
+  <si>
+    <t>0.5632890348498202</t>
+  </si>
+  <si>
+    <t>0.6317306058782529</t>
+  </si>
+  <si>
+    <t>0.7236381482984321</t>
+  </si>
+  <si>
+    <t>0.968936011904762</t>
+  </si>
+  <si>
+    <t>0.95</t>
+  </si>
+  <si>
+    <t>0.925</t>
+  </si>
+  <si>
+    <t>0.545286475232533</t>
+  </si>
+  <si>
+    <t>0.7499134164535382</t>
+  </si>
+  <si>
+    <t>0.8441762574595056</t>
+  </si>
+  <si>
+    <t>Dataset - E5 - M05 - LR000003.</t>
+  </si>
+  <si>
+    <t>0.0926499644763788</t>
+  </si>
+  <si>
+    <t>0.5582523360099181</t>
+  </si>
+  <si>
+    <t>0.9436229683659648</t>
+  </si>
+  <si>
+    <t>0.9333333333333332</t>
+  </si>
+  <si>
+    <t>0.8393333333333333</t>
+  </si>
+  <si>
+    <t>0.7710000000000004</t>
+  </si>
+  <si>
+    <t>0.5225259289419134</t>
+  </si>
+  <si>
+    <t>0.6139599674628753</t>
+  </si>
+  <si>
+    <t>0.6795462118154986</t>
+  </si>
+  <si>
+    <t>0.740563411520857</t>
+  </si>
+  <si>
+    <t>0.9485544217687074</t>
+  </si>
+  <si>
+    <t>0.903125</t>
+  </si>
+  <si>
+    <t>0.566133129111476</t>
+  </si>
+  <si>
+    <t>0.7603034420289855</t>
+  </si>
+  <si>
+    <t>0.8654624893435634</t>
+  </si>
+  <si>
+    <t>Dataset - E5 - M05 - LR00001.</t>
+  </si>
+  <si>
+    <t>0.0783674659824468</t>
+  </si>
+  <si>
+    <t>0.6262976233621287</t>
+  </si>
+  <si>
+    <t>0.9423789772899044</t>
+  </si>
+  <si>
+    <t>0.8580000000000001</t>
+  </si>
+  <si>
+    <t>0.7913333333333337</t>
+  </si>
+  <si>
+    <t>0.5666295645932315</t>
+  </si>
+  <si>
+    <t>0.6715037829964596</t>
+  </si>
+  <si>
+    <t>0.7382298604733806</t>
+  </si>
+  <si>
+    <t>0.7502549395891813</t>
+  </si>
+  <si>
+    <t>0.9391369047619048</t>
+  </si>
+  <si>
+    <t>0.915625</t>
+  </si>
+  <si>
+    <t>0.5794869760850477</t>
+  </si>
+  <si>
+    <t>0.7581588341858482</t>
+  </si>
+  <si>
+    <t>0.8356044863597613</t>
+  </si>
+  <si>
+    <t>Dataset - E5 - M06 - LR00000001.</t>
+  </si>
+  <si>
+    <t>0.913968312304696</t>
+  </si>
+  <si>
+    <t>0.4531976630359295</t>
+  </si>
+  <si>
+    <t>0.9696428571428573</t>
+  </si>
+  <si>
+    <t>0.91875</t>
+  </si>
+  <si>
+    <t>Dataset - E5 - M06 - LR0000001.</t>
+  </si>
+  <si>
+    <t>0.2807241323572745</t>
+  </si>
+  <si>
+    <t>0.3691871563837882</t>
+  </si>
+  <si>
+    <t>0.9074281565799392</t>
+  </si>
+  <si>
+    <t>0.7286666666666665</t>
+  </si>
+  <si>
+    <t>0.6420000000000005</t>
+  </si>
+  <si>
+    <t>0.3714188843010653</t>
+  </si>
+  <si>
+    <t>0.4386872460840637</t>
+  </si>
+  <si>
+    <t>0.495173836543669</t>
+  </si>
+  <si>
+    <t>0.6141074901568226</t>
+  </si>
+  <si>
+    <t>0.969758064516129</t>
+  </si>
+  <si>
+    <t>0.8875</t>
+  </si>
+  <si>
+    <t>0.4917043817040119</t>
+  </si>
+  <si>
+    <t>0.6427221906770497</t>
+  </si>
+  <si>
+    <t>0.7514915034800422</t>
+  </si>
+  <si>
+    <t>Dataset - E5 - M06 - LR000001.</t>
+  </si>
+  <si>
+    <t>0.1373885677440181</t>
+  </si>
+  <si>
+    <t>0.4922857686514711</t>
+  </si>
+  <si>
+    <t>Dataset - E5 - M06 - LR0000025.</t>
+  </si>
+  <si>
+    <t>0.1174511361403373</t>
   </si>
 </sst>
 </file>
@@ -609,25 +1242,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C267C225-13D9-4320-86DB-4969F2F2DA1A}">
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="29.4140625" customWidth="1"/>
-    <col min="2" max="2" width="19.83203125" customWidth="1"/>
-    <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="19.83203125" customWidth="1"/>
-    <col min="5" max="5" width="19.58203125" customWidth="1"/>
-    <col min="6" max="6" width="19.25" customWidth="1"/>
-    <col min="7" max="7" width="19.58203125" customWidth="1"/>
-    <col min="8" max="8" width="19.33203125" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="18.4140625" customWidth="1"/>
+    <col min="1" max="1" width="38.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.58203125" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" customWidth="1"/>
+    <col min="4" max="4" width="18.4140625" customWidth="1"/>
+    <col min="5" max="5" width="18.25" customWidth="1"/>
+    <col min="6" max="7" width="18.4140625" customWidth="1"/>
+    <col min="8" max="8" width="21.4140625" customWidth="1"/>
+    <col min="9" max="9" width="20.4140625" customWidth="1"/>
+    <col min="10" max="10" width="19.75" customWidth="1"/>
     <col min="11" max="12" width="14.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -654,7 +1286,13 @@
         <v>14</v>
       </c>
       <c r="J1" t="s">
-        <v>43</v>
+        <v>40</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
@@ -662,31 +1300,37 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="H2" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="I2" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="J2" t="s">
-        <v>45</v>
+        <v>64</v>
+      </c>
+      <c r="K2">
+        <v>300</v>
+      </c>
+      <c r="L2">
+        <v>300</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -694,33 +1338,39 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="E3" t="s">
         <v>9</v>
       </c>
       <c r="F3" t="s">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
       <c r="H3" t="s">
-        <v>27</v>
+        <v>69</v>
       </c>
       <c r="I3" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="J3" t="s">
-        <v>29</v>
+        <v>71</v>
+      </c>
+      <c r="K3">
+        <v>32</v>
+      </c>
+      <c r="L3">
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="B5" t="s">
         <v>0</v>
@@ -747,7 +1397,7 @@
         <v>14</v>
       </c>
       <c r="J5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K5" t="s">
         <v>10</v>
@@ -761,31 +1411,31 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>73</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>74</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>75</v>
       </c>
       <c r="E6" t="s">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="F6" t="s">
-        <v>19</v>
+        <v>77</v>
       </c>
       <c r="G6" t="s">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="H6" t="s">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="I6" t="s">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="J6" t="s">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="K6">
         <v>300</v>
@@ -799,28 +1449,28 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E7" t="s">
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="G7" t="s">
-        <v>26</v>
+        <v>85</v>
       </c>
       <c r="H7" t="s">
-        <v>27</v>
+        <v>86</v>
       </c>
       <c r="I7" t="s">
-        <v>28</v>
+        <v>87</v>
       </c>
       <c r="J7" t="s">
-        <v>29</v>
+        <v>88</v>
       </c>
       <c r="K7">
         <v>32</v>
@@ -831,7 +1481,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>89</v>
       </c>
       <c r="B9" t="s">
         <v>0</v>
@@ -858,7 +1508,7 @@
         <v>14</v>
       </c>
       <c r="J9" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K9" t="s">
         <v>10</v>
@@ -872,31 +1522,31 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>91</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>92</v>
       </c>
       <c r="E10" t="s">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="F10" t="s">
-        <v>33</v>
+        <v>94</v>
       </c>
       <c r="G10" t="s">
-        <v>34</v>
+        <v>95</v>
       </c>
       <c r="H10" t="s">
-        <v>35</v>
+        <v>96</v>
       </c>
       <c r="I10" t="s">
-        <v>36</v>
+        <v>97</v>
       </c>
       <c r="J10" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
       <c r="K10">
         <v>300</v>
@@ -910,28 +1560,28 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="D11" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="E11" t="s">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="F11" t="s">
-        <v>12</v>
+        <v>102</v>
       </c>
       <c r="G11" t="s">
-        <v>39</v>
+        <v>103</v>
       </c>
       <c r="H11" t="s">
-        <v>40</v>
+        <v>104</v>
       </c>
       <c r="I11" t="s">
-        <v>41</v>
+        <v>105</v>
       </c>
       <c r="J11" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="K11">
         <v>32</v>
@@ -942,7 +1592,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>67</v>
+        <v>107</v>
       </c>
       <c r="B13" t="s">
         <v>0</v>
@@ -969,7 +1619,7 @@
         <v>14</v>
       </c>
       <c r="J13" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K13" t="s">
         <v>10</v>
@@ -983,31 +1633,31 @@
         <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>51</v>
+        <v>108</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>109</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>110</v>
       </c>
       <c r="E14" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="F14" t="s">
-        <v>55</v>
+        <v>112</v>
       </c>
       <c r="G14" t="s">
-        <v>56</v>
+        <v>113</v>
       </c>
       <c r="H14" t="s">
-        <v>57</v>
+        <v>114</v>
       </c>
       <c r="I14" t="s">
-        <v>58</v>
+        <v>115</v>
       </c>
       <c r="J14" t="s">
-        <v>59</v>
+        <v>116</v>
       </c>
       <c r="K14">
         <v>300</v>
@@ -1021,28 +1671,28 @@
         <v>8</v>
       </c>
       <c r="C15" t="s">
-        <v>60</v>
+        <v>117</v>
       </c>
       <c r="D15" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
       <c r="E15" t="s">
-        <v>62</v>
+        <v>119</v>
       </c>
       <c r="F15" t="s">
-        <v>63</v>
+        <v>120</v>
       </c>
       <c r="G15" t="s">
-        <v>39</v>
+        <v>121</v>
       </c>
       <c r="H15" t="s">
-        <v>64</v>
+        <v>122</v>
       </c>
       <c r="I15" t="s">
-        <v>65</v>
+        <v>123</v>
       </c>
       <c r="J15" t="s">
-        <v>66</v>
+        <v>124</v>
       </c>
       <c r="K15">
         <v>32</v>
@@ -1053,7 +1703,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>49</v>
+        <v>125</v>
       </c>
       <c r="B17" t="s">
         <v>0</v>
@@ -1080,7 +1730,7 @@
         <v>14</v>
       </c>
       <c r="J17" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K17" t="s">
         <v>10</v>
@@ -1094,31 +1744,31 @@
         <v>7</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>126</v>
       </c>
       <c r="C18" t="s">
-        <v>16</v>
+        <v>127</v>
       </c>
       <c r="D18" t="s">
-        <v>17</v>
+        <v>128</v>
       </c>
       <c r="E18" t="s">
-        <v>18</v>
+        <v>129</v>
       </c>
       <c r="F18" t="s">
-        <v>19</v>
+        <v>130</v>
       </c>
       <c r="G18" t="s">
-        <v>20</v>
+        <v>131</v>
       </c>
       <c r="H18" t="s">
-        <v>21</v>
+        <v>132</v>
       </c>
       <c r="I18" t="s">
-        <v>22</v>
+        <v>133</v>
       </c>
       <c r="J18" t="s">
-        <v>45</v>
+        <v>134</v>
       </c>
       <c r="K18">
         <v>300</v>
@@ -1132,33 +1782,1254 @@
         <v>8</v>
       </c>
       <c r="C19" t="s">
+        <v>135</v>
+      </c>
+      <c r="D19" t="s">
+        <v>136</v>
+      </c>
+      <c r="E19" t="s">
+        <v>101</v>
+      </c>
+      <c r="F19" t="s">
+        <v>137</v>
+      </c>
+      <c r="G19" t="s">
+        <v>101</v>
+      </c>
+      <c r="H19" t="s">
+        <v>138</v>
+      </c>
+      <c r="I19" t="s">
+        <v>139</v>
+      </c>
+      <c r="J19" t="s">
+        <v>140</v>
+      </c>
+      <c r="K19">
+        <v>32</v>
+      </c>
+      <c r="L19">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>141</v>
+      </c>
+      <c r="B21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" t="s">
+        <v>1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>2</v>
+      </c>
+      <c r="E21" t="s">
+        <v>3</v>
+      </c>
+      <c r="F21" t="s">
+        <v>4</v>
+      </c>
+      <c r="G21" t="s">
+        <v>5</v>
+      </c>
+      <c r="H21" t="s">
+        <v>13</v>
+      </c>
+      <c r="I21" t="s">
+        <v>14</v>
+      </c>
+      <c r="J21" t="s">
+        <v>40</v>
+      </c>
+      <c r="K21" t="s">
+        <v>10</v>
+      </c>
+      <c r="L21" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22" t="s">
+        <v>142</v>
+      </c>
+      <c r="C22" t="s">
+        <v>143</v>
+      </c>
+      <c r="D22" t="s">
+        <v>144</v>
+      </c>
+      <c r="E22" t="s">
+        <v>145</v>
+      </c>
+      <c r="F22" t="s">
+        <v>146</v>
+      </c>
+      <c r="G22" t="s">
+        <v>147</v>
+      </c>
+      <c r="H22" t="s">
+        <v>148</v>
+      </c>
+      <c r="I22" t="s">
+        <v>149</v>
+      </c>
+      <c r="J22" t="s">
+        <v>150</v>
+      </c>
+      <c r="K22">
+        <v>300</v>
+      </c>
+      <c r="L22">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" t="s">
+        <v>151</v>
+      </c>
+      <c r="D23" t="s">
+        <v>152</v>
+      </c>
+      <c r="E23" t="s">
+        <v>9</v>
+      </c>
+      <c r="F23" t="s">
+        <v>67</v>
+      </c>
+      <c r="G23" t="s">
+        <v>153</v>
+      </c>
+      <c r="H23" t="s">
+        <v>154</v>
+      </c>
+      <c r="I23" t="s">
+        <v>155</v>
+      </c>
+      <c r="J23" t="s">
+        <v>156</v>
+      </c>
+      <c r="K23">
+        <v>32</v>
+      </c>
+      <c r="L23">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>157</v>
+      </c>
+      <c r="B25" t="s">
+        <v>0</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1</v>
+      </c>
+      <c r="D25" t="s">
+        <v>2</v>
+      </c>
+      <c r="E25" t="s">
+        <v>3</v>
+      </c>
+      <c r="F25" t="s">
+        <v>4</v>
+      </c>
+      <c r="G25" t="s">
+        <v>5</v>
+      </c>
+      <c r="H25" t="s">
+        <v>13</v>
+      </c>
+      <c r="I25" t="s">
+        <v>14</v>
+      </c>
+      <c r="J25" t="s">
+        <v>40</v>
+      </c>
+      <c r="K25" t="s">
+        <v>10</v>
+      </c>
+      <c r="L25" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" t="s">
+        <v>158</v>
+      </c>
+      <c r="C26" t="s">
+        <v>159</v>
+      </c>
+      <c r="D26" t="s">
+        <v>160</v>
+      </c>
+      <c r="E26" t="s">
+        <v>161</v>
+      </c>
+      <c r="F26" t="s">
+        <v>162</v>
+      </c>
+      <c r="G26" t="s">
+        <v>163</v>
+      </c>
+      <c r="H26" t="s">
+        <v>164</v>
+      </c>
+      <c r="I26" t="s">
+        <v>165</v>
+      </c>
+      <c r="J26" t="s">
+        <v>166</v>
+      </c>
+      <c r="K26">
+        <v>300</v>
+      </c>
+      <c r="L26">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" t="s">
+        <v>167</v>
+      </c>
+      <c r="D27" t="s">
+        <v>168</v>
+      </c>
+      <c r="E27" t="s">
+        <v>101</v>
+      </c>
+      <c r="F27" t="s">
+        <v>101</v>
+      </c>
+      <c r="G27" t="s">
+        <v>169</v>
+      </c>
+      <c r="H27" t="s">
+        <v>170</v>
+      </c>
+      <c r="I27" t="s">
+        <v>171</v>
+      </c>
+      <c r="J27" t="s">
+        <v>172</v>
+      </c>
+      <c r="K27">
+        <v>32</v>
+      </c>
+      <c r="L27">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>173</v>
+      </c>
+      <c r="B29" t="s">
+        <v>0</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1</v>
+      </c>
+      <c r="D29" t="s">
+        <v>2</v>
+      </c>
+      <c r="E29" t="s">
+        <v>3</v>
+      </c>
+      <c r="F29" t="s">
+        <v>4</v>
+      </c>
+      <c r="G29" t="s">
+        <v>5</v>
+      </c>
+      <c r="H29" t="s">
+        <v>13</v>
+      </c>
+      <c r="I29" t="s">
+        <v>14</v>
+      </c>
+      <c r="J29" t="s">
+        <v>40</v>
+      </c>
+      <c r="K29" t="s">
+        <v>10</v>
+      </c>
+      <c r="L29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" t="s">
+        <v>174</v>
+      </c>
+      <c r="C30" t="s">
+        <v>175</v>
+      </c>
+      <c r="D30" t="s">
+        <v>176</v>
+      </c>
+      <c r="E30" t="s">
+        <v>177</v>
+      </c>
+      <c r="F30" t="s">
+        <v>178</v>
+      </c>
+      <c r="G30" t="s">
+        <v>179</v>
+      </c>
+      <c r="H30" t="s">
+        <v>180</v>
+      </c>
+      <c r="I30" t="s">
+        <v>181</v>
+      </c>
+      <c r="J30" t="s">
+        <v>182</v>
+      </c>
+      <c r="K30">
+        <v>300</v>
+      </c>
+      <c r="L30">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" t="s">
+        <v>183</v>
+      </c>
+      <c r="D31" t="s">
+        <v>184</v>
+      </c>
+      <c r="E31" t="s">
+        <v>51</v>
+      </c>
+      <c r="F31" t="s">
+        <v>185</v>
+      </c>
+      <c r="G31" t="s">
+        <v>186</v>
+      </c>
+      <c r="H31" t="s">
+        <v>187</v>
+      </c>
+      <c r="I31" t="s">
+        <v>188</v>
+      </c>
+      <c r="J31" t="s">
+        <v>189</v>
+      </c>
+      <c r="K31">
+        <v>32</v>
+      </c>
+      <c r="L31">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>190</v>
+      </c>
+      <c r="B33" t="s">
+        <v>0</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1</v>
+      </c>
+      <c r="D33" t="s">
+        <v>2</v>
+      </c>
+      <c r="E33" t="s">
+        <v>3</v>
+      </c>
+      <c r="F33" t="s">
+        <v>4</v>
+      </c>
+      <c r="G33" t="s">
+        <v>5</v>
+      </c>
+      <c r="H33" t="s">
+        <v>13</v>
+      </c>
+      <c r="I33" t="s">
+        <v>14</v>
+      </c>
+      <c r="J33" t="s">
+        <v>40</v>
+      </c>
+      <c r="K33" t="s">
+        <v>10</v>
+      </c>
+      <c r="L33" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" t="s">
+        <v>191</v>
+      </c>
+      <c r="C34" t="s">
+        <v>192</v>
+      </c>
+      <c r="D34" t="s">
+        <v>193</v>
+      </c>
+      <c r="E34" t="s">
+        <v>194</v>
+      </c>
+      <c r="F34" t="s">
+        <v>195</v>
+      </c>
+      <c r="G34" t="s">
+        <v>196</v>
+      </c>
+      <c r="H34" t="s">
+        <v>197</v>
+      </c>
+      <c r="I34" t="s">
+        <v>198</v>
+      </c>
+      <c r="J34" t="s">
+        <v>199</v>
+      </c>
+      <c r="K34">
+        <v>300</v>
+      </c>
+      <c r="L34">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35" t="s">
+        <v>200</v>
+      </c>
+      <c r="D35" t="s">
+        <v>201</v>
+      </c>
+      <c r="E35" t="s">
+        <v>12</v>
+      </c>
+      <c r="F35" t="s">
+        <v>202</v>
+      </c>
+      <c r="G35" t="s">
+        <v>203</v>
+      </c>
+      <c r="H35" t="s">
+        <v>204</v>
+      </c>
+      <c r="I35" t="s">
+        <v>205</v>
+      </c>
+      <c r="J35" t="s">
+        <v>206</v>
+      </c>
+      <c r="K35">
+        <v>32</v>
+      </c>
+      <c r="L35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>207</v>
+      </c>
+      <c r="B37" t="s">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1</v>
+      </c>
+      <c r="D37" t="s">
+        <v>2</v>
+      </c>
+      <c r="E37" t="s">
+        <v>3</v>
+      </c>
+      <c r="F37" t="s">
+        <v>4</v>
+      </c>
+      <c r="G37" t="s">
+        <v>5</v>
+      </c>
+      <c r="H37" t="s">
+        <v>13</v>
+      </c>
+      <c r="I37" t="s">
+        <v>14</v>
+      </c>
+      <c r="J37" t="s">
+        <v>40</v>
+      </c>
+      <c r="K37" t="s">
+        <v>10</v>
+      </c>
+      <c r="L37" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>7</v>
+      </c>
+      <c r="B38" t="s">
+        <v>208</v>
+      </c>
+      <c r="C38" t="s">
+        <v>209</v>
+      </c>
+      <c r="D38" t="s">
+        <v>210</v>
+      </c>
+      <c r="E38" t="s">
+        <v>59</v>
+      </c>
+      <c r="F38" t="s">
+        <v>211</v>
+      </c>
+      <c r="G38" t="s">
+        <v>212</v>
+      </c>
+      <c r="H38" t="s">
+        <v>213</v>
+      </c>
+      <c r="I38" t="s">
+        <v>214</v>
+      </c>
+      <c r="J38" t="s">
+        <v>215</v>
+      </c>
+      <c r="K38">
+        <v>300</v>
+      </c>
+      <c r="L38">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39" t="s">
+        <v>216</v>
+      </c>
+      <c r="D39" t="s">
+        <v>217</v>
+      </c>
+      <c r="E39" t="s">
+        <v>51</v>
+      </c>
+      <c r="F39" t="s">
+        <v>218</v>
+      </c>
+      <c r="G39" t="s">
+        <v>219</v>
+      </c>
+      <c r="H39" t="s">
+        <v>220</v>
+      </c>
+      <c r="I39" t="s">
+        <v>221</v>
+      </c>
+      <c r="J39" t="s">
+        <v>222</v>
+      </c>
+      <c r="K39">
+        <v>32</v>
+      </c>
+      <c r="L39">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>223</v>
+      </c>
+      <c r="B41" t="s">
+        <v>0</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1</v>
+      </c>
+      <c r="D41" t="s">
+        <v>2</v>
+      </c>
+      <c r="E41" t="s">
+        <v>3</v>
+      </c>
+      <c r="F41" t="s">
+        <v>4</v>
+      </c>
+      <c r="G41" t="s">
+        <v>5</v>
+      </c>
+      <c r="H41" t="s">
+        <v>13</v>
+      </c>
+      <c r="I41" t="s">
+        <v>14</v>
+      </c>
+      <c r="J41" t="s">
+        <v>40</v>
+      </c>
+      <c r="K41" t="s">
+        <v>10</v>
+      </c>
+      <c r="L41" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42" t="s">
+        <v>224</v>
+      </c>
+      <c r="C42" t="s">
+        <v>225</v>
+      </c>
+      <c r="D42" t="s">
+        <v>226</v>
+      </c>
+      <c r="E42" t="s">
+        <v>227</v>
+      </c>
+      <c r="F42" t="s">
+        <v>228</v>
+      </c>
+      <c r="G42" t="s">
+        <v>229</v>
+      </c>
+      <c r="H42" t="s">
+        <v>230</v>
+      </c>
+      <c r="I42" t="s">
+        <v>231</v>
+      </c>
+      <c r="J42" t="s">
+        <v>232</v>
+      </c>
+      <c r="K42">
+        <v>300</v>
+      </c>
+      <c r="L42">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" t="s">
+        <v>233</v>
+      </c>
+      <c r="D43" t="s">
+        <v>234</v>
+      </c>
+      <c r="E43" t="s">
+        <v>12</v>
+      </c>
+      <c r="F43" t="s">
+        <v>219</v>
+      </c>
+      <c r="G43" t="s">
+        <v>235</v>
+      </c>
+      <c r="H43" t="s">
+        <v>236</v>
+      </c>
+      <c r="I43" t="s">
+        <v>237</v>
+      </c>
+      <c r="J43" t="s">
+        <v>238</v>
+      </c>
+      <c r="K43">
+        <v>32</v>
+      </c>
+      <c r="L43">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>239</v>
+      </c>
+      <c r="B45" t="s">
+        <v>0</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1</v>
+      </c>
+      <c r="D45" t="s">
+        <v>2</v>
+      </c>
+      <c r="E45" t="s">
+        <v>3</v>
+      </c>
+      <c r="F45" t="s">
+        <v>4</v>
+      </c>
+      <c r="G45" t="s">
+        <v>5</v>
+      </c>
+      <c r="H45" t="s">
+        <v>13</v>
+      </c>
+      <c r="I45" t="s">
+        <v>14</v>
+      </c>
+      <c r="J45" t="s">
+        <v>40</v>
+      </c>
+      <c r="K45" t="s">
+        <v>10</v>
+      </c>
+      <c r="L45" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>7</v>
+      </c>
+      <c r="B46" t="s">
+        <v>240</v>
+      </c>
+      <c r="C46" t="s">
+        <v>241</v>
+      </c>
+      <c r="D46" t="s">
+        <v>242</v>
+      </c>
+      <c r="E46" t="s">
+        <v>11</v>
+      </c>
+      <c r="F46" t="s">
+        <v>243</v>
+      </c>
+      <c r="G46" t="s">
+        <v>244</v>
+      </c>
+      <c r="H46" t="s">
+        <v>245</v>
+      </c>
+      <c r="I46" t="s">
+        <v>246</v>
+      </c>
+      <c r="J46" t="s">
+        <v>247</v>
+      </c>
+      <c r="K46">
+        <v>300</v>
+      </c>
+      <c r="L46">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>8</v>
+      </c>
+      <c r="C47" t="s">
+        <v>248</v>
+      </c>
+      <c r="D47" t="s">
+        <v>249</v>
+      </c>
+      <c r="E47" t="s">
+        <v>12</v>
+      </c>
+      <c r="F47" t="s">
+        <v>185</v>
+      </c>
+      <c r="G47" t="s">
+        <v>250</v>
+      </c>
+      <c r="H47" t="s">
+        <v>251</v>
+      </c>
+      <c r="I47" t="s">
+        <v>252</v>
+      </c>
+      <c r="J47" t="s">
+        <v>253</v>
+      </c>
+      <c r="K47">
+        <v>32</v>
+      </c>
+      <c r="L47">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>254</v>
+      </c>
+      <c r="B49" t="s">
+        <v>0</v>
+      </c>
+      <c r="C49" t="s">
+        <v>1</v>
+      </c>
+      <c r="D49" t="s">
+        <v>2</v>
+      </c>
+      <c r="E49" t="s">
+        <v>3</v>
+      </c>
+      <c r="F49" t="s">
+        <v>4</v>
+      </c>
+      <c r="G49" t="s">
+        <v>5</v>
+      </c>
+      <c r="H49" t="s">
+        <v>13</v>
+      </c>
+      <c r="I49" t="s">
+        <v>14</v>
+      </c>
+      <c r="J49" t="s">
+        <v>40</v>
+      </c>
+      <c r="K49" t="s">
+        <v>10</v>
+      </c>
+      <c r="L49" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>7</v>
+      </c>
+      <c r="B50" t="s">
+        <v>43</v>
+      </c>
+      <c r="C50" t="s">
+        <v>44</v>
+      </c>
+      <c r="D50" t="s">
+        <v>255</v>
+      </c>
+      <c r="E50" t="s">
+        <v>45</v>
+      </c>
+      <c r="F50" t="s">
+        <v>46</v>
+      </c>
+      <c r="G50" t="s">
+        <v>47</v>
+      </c>
+      <c r="H50" t="s">
+        <v>48</v>
+      </c>
+      <c r="I50" t="s">
+        <v>256</v>
+      </c>
+      <c r="J50" t="s">
+        <v>49</v>
+      </c>
+      <c r="K50">
+        <v>300</v>
+      </c>
+      <c r="L50">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51" t="s">
+        <v>50</v>
+      </c>
+      <c r="D51" t="s">
+        <v>257</v>
+      </c>
+      <c r="E51" t="s">
+        <v>51</v>
+      </c>
+      <c r="F51" t="s">
+        <v>258</v>
+      </c>
+      <c r="G51" t="s">
+        <v>36</v>
+      </c>
+      <c r="H51" t="s">
+        <v>52</v>
+      </c>
+      <c r="I51" t="s">
+        <v>53</v>
+      </c>
+      <c r="J51" t="s">
+        <v>54</v>
+      </c>
+      <c r="K51">
+        <v>32</v>
+      </c>
+      <c r="L51">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>259</v>
+      </c>
+      <c r="B53" t="s">
+        <v>0</v>
+      </c>
+      <c r="C53" t="s">
+        <v>1</v>
+      </c>
+      <c r="D53" t="s">
+        <v>2</v>
+      </c>
+      <c r="E53" t="s">
+        <v>3</v>
+      </c>
+      <c r="F53" t="s">
+        <v>4</v>
+      </c>
+      <c r="G53" t="s">
+        <v>5</v>
+      </c>
+      <c r="H53" t="s">
+        <v>13</v>
+      </c>
+      <c r="I53" t="s">
+        <v>14</v>
+      </c>
+      <c r="J53" t="s">
+        <v>40</v>
+      </c>
+      <c r="K53" t="s">
+        <v>10</v>
+      </c>
+      <c r="L53" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>7</v>
+      </c>
+      <c r="B54" t="s">
+        <v>260</v>
+      </c>
+      <c r="C54" t="s">
+        <v>261</v>
+      </c>
+      <c r="D54" t="s">
+        <v>262</v>
+      </c>
+      <c r="E54" t="s">
+        <v>177</v>
+      </c>
+      <c r="F54" t="s">
+        <v>263</v>
+      </c>
+      <c r="G54" t="s">
+        <v>264</v>
+      </c>
+      <c r="H54" t="s">
+        <v>265</v>
+      </c>
+      <c r="I54" t="s">
+        <v>266</v>
+      </c>
+      <c r="J54" t="s">
+        <v>267</v>
+      </c>
+      <c r="K54">
+        <v>300</v>
+      </c>
+      <c r="L54">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>8</v>
+      </c>
+      <c r="C55" t="s">
+        <v>268</v>
+      </c>
+      <c r="D55" t="s">
+        <v>269</v>
+      </c>
+      <c r="E55" t="s">
+        <v>51</v>
+      </c>
+      <c r="F55" t="s">
+        <v>258</v>
+      </c>
+      <c r="G55" t="s">
+        <v>270</v>
+      </c>
+      <c r="H55" t="s">
+        <v>271</v>
+      </c>
+      <c r="I55" t="s">
+        <v>272</v>
+      </c>
+      <c r="J55" t="s">
+        <v>273</v>
+      </c>
+      <c r="K55">
+        <v>32</v>
+      </c>
+      <c r="L55">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>274</v>
+      </c>
+      <c r="B57" t="s">
+        <v>0</v>
+      </c>
+      <c r="C57" t="s">
+        <v>1</v>
+      </c>
+      <c r="D57" t="s">
+        <v>2</v>
+      </c>
+      <c r="E57" t="s">
+        <v>3</v>
+      </c>
+      <c r="F57" t="s">
+        <v>4</v>
+      </c>
+      <c r="G57" t="s">
+        <v>5</v>
+      </c>
+      <c r="H57" t="s">
+        <v>13</v>
+      </c>
+      <c r="I57" t="s">
+        <v>14</v>
+      </c>
+      <c r="J57" t="s">
+        <v>40</v>
+      </c>
+      <c r="K57" t="s">
+        <v>10</v>
+      </c>
+      <c r="L57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>7</v>
+      </c>
+      <c r="B58" t="s">
+        <v>275</v>
+      </c>
+      <c r="C58" t="s">
+        <v>29</v>
+      </c>
+      <c r="D58" t="s">
+        <v>30</v>
+      </c>
+      <c r="E58" t="s">
+        <v>11</v>
+      </c>
+      <c r="F58" t="s">
+        <v>31</v>
+      </c>
+      <c r="G58" t="s">
+        <v>32</v>
+      </c>
+      <c r="H58" t="s">
+        <v>276</v>
+      </c>
+      <c r="I58" t="s">
+        <v>33</v>
+      </c>
+      <c r="J58" t="s">
+        <v>42</v>
+      </c>
+      <c r="K58">
+        <v>300</v>
+      </c>
+      <c r="L58">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>8</v>
+      </c>
+      <c r="C59" t="s">
+        <v>34</v>
+      </c>
+      <c r="D59" t="s">
+        <v>35</v>
+      </c>
+      <c r="E59" t="s">
+        <v>12</v>
+      </c>
+      <c r="F59" t="s">
+        <v>12</v>
+      </c>
+      <c r="G59" t="s">
+        <v>36</v>
+      </c>
+      <c r="H59" t="s">
+        <v>37</v>
+      </c>
+      <c r="I59" t="s">
+        <v>38</v>
+      </c>
+      <c r="J59" t="s">
+        <v>39</v>
+      </c>
+      <c r="K59">
+        <v>32</v>
+      </c>
+      <c r="L59">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>277</v>
+      </c>
+      <c r="B61" t="s">
+        <v>0</v>
+      </c>
+      <c r="C61" t="s">
+        <v>1</v>
+      </c>
+      <c r="D61" t="s">
+        <v>2</v>
+      </c>
+      <c r="E61" t="s">
+        <v>3</v>
+      </c>
+      <c r="F61" t="s">
+        <v>4</v>
+      </c>
+      <c r="G61" t="s">
+        <v>5</v>
+      </c>
+      <c r="H61" t="s">
+        <v>13</v>
+      </c>
+      <c r="I61" t="s">
+        <v>14</v>
+      </c>
+      <c r="J61" t="s">
+        <v>40</v>
+      </c>
+      <c r="K61" t="s">
+        <v>10</v>
+      </c>
+      <c r="L61" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>7</v>
+      </c>
+      <c r="B62" t="s">
+        <v>278</v>
+      </c>
+      <c r="C62" t="s">
+        <v>15</v>
+      </c>
+      <c r="D62" t="s">
+        <v>16</v>
+      </c>
+      <c r="E62" t="s">
+        <v>17</v>
+      </c>
+      <c r="F62" t="s">
+        <v>18</v>
+      </c>
+      <c r="G62" t="s">
+        <v>19</v>
+      </c>
+      <c r="H62" t="s">
+        <v>20</v>
+      </c>
+      <c r="I62" t="s">
+        <v>21</v>
+      </c>
+      <c r="J62" t="s">
+        <v>41</v>
+      </c>
+      <c r="K62">
+        <v>300</v>
+      </c>
+      <c r="L62">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>8</v>
+      </c>
+      <c r="C63" t="s">
+        <v>22</v>
+      </c>
+      <c r="D63" t="s">
         <v>23</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E63" t="s">
+        <v>9</v>
+      </c>
+      <c r="F63" t="s">
         <v>24</v>
       </c>
-      <c r="E19" t="s">
-        <v>9</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="G63" t="s">
         <v>25</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H63" t="s">
         <v>26</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I63" t="s">
         <v>27</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J63" t="s">
         <v>28</v>
       </c>
-      <c r="J19" t="s">
-        <v>29</v>
-      </c>
-      <c r="K19">
-        <v>32</v>
-      </c>
-      <c r="L19">
+      <c r="K63">
+        <v>32</v>
+      </c>
+      <c r="L63">
         <v>32</v>
       </c>
     </row>
@@ -1169,28 +3040,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A28"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="2" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="3" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="6" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="7" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="8" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="11" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="12" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="13" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="16" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="17" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="18" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="21" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="22" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="23" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="26" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="27" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="28" ht="15.5" x14ac:dyDescent="0.35"/>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>